<commit_message>
Simple chatBot deposit filtering, no Hebrew support yet, Some fetures are missing still
</commit_message>
<xml_diff>
--- a/data/seed/bank_deposits.xlsx
+++ b/data/seed/bank_deposits.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,14 +707,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>99-888-777001</t>
+          <t>12-345-678902</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46032</v>
+        <v>46086</v>
       </c>
       <c r="C11" t="n">
-        <v>4800</v>
+        <v>6200</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -723,12 +723,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DEP-2026-010</t>
+          <t>DEP-2026-016</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Owner deposit - January</t>
+          <t>Owner deposit - March</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46063</v>
+        <v>46032</v>
       </c>
       <c r="C12" t="n">
         <v>4800</v>
@@ -751,12 +751,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>DEP-2026-011</t>
+          <t>DEP-2026-010</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Owner deposit - February</t>
+          <t>Owner deposit - January</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46091</v>
+        <v>46063</v>
       </c>
       <c r="C13" t="n">
         <v>4800</v>
@@ -779,12 +779,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DEP-2026-012</t>
+          <t>DEP-2026-011</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Owner deposit - March</t>
+          <t>Owner deposit - February</t>
         </is>
       </c>
     </row>
@@ -795,10 +795,10 @@
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46106</v>
+        <v>46091</v>
       </c>
       <c r="C14" t="n">
-        <v>300</v>
+        <v>4800</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -807,12 +807,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DEP-2026-013</t>
+          <t>DEP-2026-012</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Insurance refund</t>
+          <t>Owner deposit - March</t>
         </is>
       </c>
     </row>
@@ -823,10 +823,10 @@
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46122</v>
+        <v>46106</v>
       </c>
       <c r="C15" t="n">
-        <v>4800</v>
+        <v>300</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -835,12 +835,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>DEP-2026-014</t>
+          <t>DEP-2026-013</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Owner deposit - April</t>
+          <t>Insurance refund</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46152</v>
+        <v>46122</v>
       </c>
       <c r="C16" t="n">
         <v>4800</v>
@@ -863,12 +863,68 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>DEP-2026-014</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Owner deposit - April</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>99-888-777001</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46152</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4800</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>DEP-2026-015</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Owner deposit - May</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>12-345-678901</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C18" t="n">
+        <v>8500</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DEP-2026-017</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Owner deposit - June</t>
         </is>
       </c>
     </row>

</xml_diff>